<commit_message>
Republish the guide from the terminology updates and add the September 2026 non-artifact pages redline.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/ValueSet-ahip-background-asian-category.xlsx
+++ b/docs/ValueSet-ahip-background-asian-category.xlsx
@@ -95,7 +95,9 @@
     <t>Copyright</t>
   </si>
   <si>
-    <t>Used by permission of HL7 International, all rights reserved Creative Commons License</t>
+    <t>Most of the information on the CDC and ATSDR websites is not subject to copyright, is in the public domain, and may be freely used or reproduced without obtaining copyright permission. For information and exceptions regarding use of CDC material please see https://www.cdc.gov/other/agencymaterials.html.
+This material derives from the HL7 Terminology (THO). THO is copyright ©1989+ Health Level Seven International and is made available under the CC0 designation. For more licensing information see: https://terminology.hl7.org/license.html
+This value set includes content developed through the DEMo Initiative and is subject to joint copyright of America's Health Insurance Plans (AHIP) and Health Level Seven International (HL7).</t>
   </si>
   <si>
     <t>Immutable</t>
@@ -230,7 +232,7 @@
     <t>I choose not to respond at this time</t>
   </si>
   <si>
-    <t>http://ahip.org/demographics/CodeSystem/AHIP-Demo-Additional-NullFlavor</t>
+    <t>http://ahip.org/demographics/CodeSystem/ahip-demo-additional-nullFlavor</t>
   </si>
 </sst>
 </file>

</xml_diff>